<commit_message>
Update to script and figure 4
</commit_message>
<xml_diff>
--- a/Scripts R/AIC valuation models.xlsx
+++ b/Scripts R/AIC valuation models.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Mi unidad\2025\SnowFire\Scripts R\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20F2D236-C0A8-46D4-861D-33F49C3A35BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5393EB46-2503-4E23-89F6-F1C56E133616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24660" yWindow="1310" windowWidth="28800" windowHeight="15410" xr2:uid="{07AB2F92-461C-495A-B893-E7D41FE87EF8}"/>
+    <workbookView xWindow="24660" yWindow="1310" windowWidth="28800" windowHeight="15410" activeTab="3" xr2:uid="{07AB2F92-461C-495A-B893-E7D41FE87EF8}"/>
   </bookViews>
   <sheets>
-    <sheet name="Pre fire" sheetId="2" r:id="rId1"/>
-    <sheet name="Post fire" sheetId="1" r:id="rId2"/>
+    <sheet name="Hoja1" sheetId="3" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="4" r:id="rId2"/>
+    <sheet name="Pre fire" sheetId="2" r:id="rId3"/>
+    <sheet name="Post fire" sheetId="1" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="86">
   <si>
     <t>Step</t>
   </si>
@@ -143,13 +145,163 @@
   </si>
   <si>
     <t>Snow occurrence (%) ~ Elevation + Longitude + Treatment + Latitude + Curvature + Slope + Orientation + Shadows</t>
+  </si>
+  <si>
+    <t>===============================================</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                    Dependent variable:        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">             ----------------------------------</t>
+  </si>
+  <si>
+    <t xml:space="preserve">             Percentage of snow occurrence (%) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">                 Pre-fire         Post-fire    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">                    (1)              (2)       </t>
+  </si>
+  <si>
+    <t>-----------------------------------------------</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PCL              -5.956***        -15.835***   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">                  (0.957)          (0.909)     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SL                2.434*          -10.501***   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">                  (1.307)          (1.167)     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Curvature                          0.028***    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insolation                        -59.075**    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slope                              0.251***    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orientation      0.151***           0.062      </t>
+  </si>
+  <si>
+    <t xml:space="preserve">                  (0.015)          (0.040)     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shadows          -0.020***          0.013      </t>
+  </si>
+  <si>
+    <t xml:space="preserve">                  (0.004)          (0.010)     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">x                -0.038***                     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">y                -0.152***        -0.443***    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">                  (0.041)          (0.162)     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intercept                           0.642      </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Constant       9,104.939***    -121,194.900*** </t>
+  </si>
+  <si>
+    <t xml:space="preserve">                (1,600.878)      (29,168.040)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observations        422              422       </t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2                 0.482            0.810      </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adjusted R2        0.474            0.806      </t>
+  </si>
+  <si>
+    <t>Note:               *p&lt;0.1; **p&lt;0.05; ***p&lt;0.01</t>
+  </si>
+  <si>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>Estimate</t>
+  </si>
+  <si>
+    <t>Std. Error</t>
+  </si>
+  <si>
+    <t>t value</t>
+  </si>
+  <si>
+    <t>p value</t>
+  </si>
+  <si>
+    <t>&lt;0.01</t>
+  </si>
+  <si>
+    <t>PCL</t>
+  </si>
+  <si>
+    <t>SL</t>
+  </si>
+  <si>
+    <t>&lt;0.1</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
+  <si>
+    <t>(Intercept)</t>
+  </si>
+  <si>
+    <t>n.s.</t>
+  </si>
+  <si>
+    <t>&lt;0.05</t>
+  </si>
+  <si>
+    <t>Pre fire period</t>
+  </si>
+  <si>
+    <t>Post fire period</t>
+  </si>
+  <si>
+    <t>Period</t>
+  </si>
+  <si>
+    <t>Pre-fire</t>
+  </si>
+  <si>
+    <t>Post-fire</t>
+  </si>
+  <si>
+    <t>Treatment_SL</t>
+  </si>
+  <si>
+    <t>Treatment_PCL</t>
+  </si>
+  <si>
+    <t>&lt;0.0001</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -175,6 +327,14 @@
       <color rgb="FFFFFFFF"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -223,7 +383,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -239,6 +399,15 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -553,6 +722,787 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACAE188C-E84B-4EA4-BB49-AF8DBE356CDB}">
+  <dimension ref="A1:L35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" t="s">
+        <v>78</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="I3" s="7">
+        <v>-5.9560000000000004</v>
+      </c>
+      <c r="J3" s="7">
+        <v>0.95699999999999996</v>
+      </c>
+      <c r="K3" s="7">
+        <v>-6.226</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="I4" s="7">
+        <v>2.4340000000000002</v>
+      </c>
+      <c r="J4" s="7">
+        <v>1.3069999999999999</v>
+      </c>
+      <c r="K4" s="7">
+        <v>1.863</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>40</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="7">
+        <v>0.151</v>
+      </c>
+      <c r="J5" s="7">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="K5" s="7">
+        <v>10.067</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>41</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="I6" s="7">
+        <v>-0.02</v>
+      </c>
+      <c r="J6" s="7">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="K6" s="7">
+        <v>-5</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="I7" s="7">
+        <v>-3.7999999999999999E-2</v>
+      </c>
+      <c r="J7" s="7">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="K7" s="7">
+        <v>-4.2220000000000004</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>43</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="I8" s="7">
+        <v>-0.152</v>
+      </c>
+      <c r="J8" s="7">
+        <v>4.1000000000000002E-2</v>
+      </c>
+      <c r="K8" s="7">
+        <v>-3.7069999999999999</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>44</v>
+      </c>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="6"/>
+      <c r="L9" s="6"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>45</v>
+      </c>
+      <c r="G10" t="s">
+        <v>79</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="I10" s="7">
+        <v>0.64200000000000002</v>
+      </c>
+      <c r="J10" s="7">
+        <v>0.41099999999999998</v>
+      </c>
+      <c r="K10" s="7">
+        <v>1.5629999999999999</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>46</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="I11" s="7">
+        <v>-15.835000000000001</v>
+      </c>
+      <c r="J11" s="7">
+        <v>0.90900000000000003</v>
+      </c>
+      <c r="K11" s="7">
+        <v>-17.425999999999998</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>47</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="I12" s="7">
+        <v>-10.500999999999999</v>
+      </c>
+      <c r="J12" s="7">
+        <v>1.167</v>
+      </c>
+      <c r="K12" s="7">
+        <v>-9.0009999999999994</v>
+      </c>
+      <c r="L12" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>-6.0000000000000001E-3</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="I13" s="7">
+        <v>2.8000000000000001E-2</v>
+      </c>
+      <c r="J13" s="7">
+        <v>6.0000000000000001E-3</v>
+      </c>
+      <c r="K13" s="7">
+        <v>4.6669999999999998</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>48</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I14" s="7">
+        <v>-59.075000000000003</v>
+      </c>
+      <c r="J14" s="7">
+        <v>27.978000000000002</v>
+      </c>
+      <c r="K14" s="7">
+        <v>-2.1120000000000001</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>-27.978000000000002</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I15" s="7">
+        <v>0.251</v>
+      </c>
+      <c r="J15" s="7">
+        <v>8.1000000000000003E-2</v>
+      </c>
+      <c r="K15" s="7">
+        <v>3.0990000000000002</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>49</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="I16" s="7">
+        <v>6.2E-2</v>
+      </c>
+      <c r="J16" s="7">
+        <v>0.04</v>
+      </c>
+      <c r="K16" s="7">
+        <v>1.55</v>
+      </c>
+      <c r="L16" s="7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>-8.1000000000000003E-2</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="I17" s="7">
+        <v>1.2999999999999999E-2</v>
+      </c>
+      <c r="J17" s="7">
+        <v>0.01</v>
+      </c>
+      <c r="K17" s="7">
+        <v>1.3</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>50</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="I18" s="7">
+        <v>-0.443</v>
+      </c>
+      <c r="J18" s="7">
+        <v>0.16200000000000001</v>
+      </c>
+      <c r="K18" s="7">
+        <v>-2.7360000000000002</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>51</v>
+      </c>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
+      <c r="J19" s="7"/>
+      <c r="K19" s="7"/>
+      <c r="L19" s="7"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>-8.9999999999999993E-3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>-0.41099999999999998</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B19244A-F6C2-4CDB-AED9-39A128AEB35B}">
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="17.88671875" customWidth="1"/>
+    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2">
+        <v>9105</v>
+      </c>
+      <c r="D2">
+        <v>1601</v>
+      </c>
+      <c r="E2">
+        <v>5.6870000000000003</v>
+      </c>
+      <c r="F2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C3">
+        <v>-5.9560000000000004</v>
+      </c>
+      <c r="D3">
+        <v>0.95669999999999999</v>
+      </c>
+      <c r="E3">
+        <v>-6.226</v>
+      </c>
+      <c r="F3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4">
+        <v>2.4340000000000002</v>
+      </c>
+      <c r="D4">
+        <v>1.3069999999999999</v>
+      </c>
+      <c r="E4">
+        <v>1.8620000000000001</v>
+      </c>
+      <c r="F4">
+        <v>6.3249E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5">
+        <v>0.1512</v>
+      </c>
+      <c r="D5">
+        <v>1.452E-2</v>
+      </c>
+      <c r="E5">
+        <v>10.411</v>
+      </c>
+      <c r="F5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6">
+        <v>-2.0279999999999999E-2</v>
+      </c>
+      <c r="D6">
+        <v>3.5560000000000001E-3</v>
+      </c>
+      <c r="E6">
+        <v>-5.702</v>
+      </c>
+      <c r="F6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7">
+        <v>-3.8109999999999998E-2</v>
+      </c>
+      <c r="D7">
+        <v>8.6029999999999995E-3</v>
+      </c>
+      <c r="E7">
+        <v>-4.43</v>
+      </c>
+      <c r="F7" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8">
+        <v>-0.15160000000000001</v>
+      </c>
+      <c r="D8">
+        <v>4.0770000000000001E-2</v>
+      </c>
+      <c r="E8">
+        <v>-3.718</v>
+      </c>
+      <c r="F8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>82</v>
+      </c>
+      <c r="B9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C9">
+        <v>-121200</v>
+      </c>
+      <c r="D9">
+        <v>29170</v>
+      </c>
+      <c r="E9">
+        <v>-4.1550000000000002</v>
+      </c>
+      <c r="F9" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10">
+        <v>6.2019999999999999E-2</v>
+      </c>
+      <c r="D10">
+        <v>4.045E-2</v>
+      </c>
+      <c r="E10">
+        <v>1.534</v>
+      </c>
+      <c r="F10">
+        <v>0.12590999999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11">
+        <v>1.2579999999999999E-2</v>
+      </c>
+      <c r="D11">
+        <v>0.01</v>
+      </c>
+      <c r="E11">
+        <v>1.258</v>
+      </c>
+      <c r="F11">
+        <v>0.20896999999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B12" t="s">
+        <v>84</v>
+      </c>
+      <c r="C12">
+        <v>-15.83</v>
+      </c>
+      <c r="D12">
+        <v>0.90900000000000003</v>
+      </c>
+      <c r="E12">
+        <v>-17.420999999999999</v>
+      </c>
+      <c r="F12" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C13">
+        <v>-10.5</v>
+      </c>
+      <c r="D13">
+        <v>1.167</v>
+      </c>
+      <c r="E13">
+        <v>-8.9969999999999999</v>
+      </c>
+      <c r="F13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14">
+        <v>2.8199999999999999E-2</v>
+      </c>
+      <c r="D14">
+        <v>6.0889999999999998E-3</v>
+      </c>
+      <c r="E14">
+        <v>4.63</v>
+      </c>
+      <c r="F14" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15">
+        <v>-59.07</v>
+      </c>
+      <c r="D15">
+        <v>27.98</v>
+      </c>
+      <c r="E15">
+        <v>-2.1120000000000001</v>
+      </c>
+      <c r="F15">
+        <v>3.533E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16">
+        <v>0.25090000000000001</v>
+      </c>
+      <c r="D16">
+        <v>8.0610000000000001E-2</v>
+      </c>
+      <c r="E16">
+        <v>3.113</v>
+      </c>
+      <c r="F16" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17">
+        <v>-0.44259999999999999</v>
+      </c>
+      <c r="D17">
+        <v>0.16220000000000001</v>
+      </c>
+      <c r="E17">
+        <v>-2.7280000000000002</v>
+      </c>
+      <c r="F17">
+        <v>6.6400000000000001E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="7"/>
+      <c r="B18" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="8">
+        <v>0.6421</v>
+      </c>
+      <c r="D18" s="8">
+        <v>0.41120000000000001</v>
+      </c>
+      <c r="E18" s="8">
+        <v>1.5620000000000001</v>
+      </c>
+      <c r="F18" s="8">
+        <v>0.11914</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF43A57F-32D7-4469-9CF0-D3F489CE9B6F}">
   <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -733,7 +1683,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3543F4B8-D571-4E28-91A6-4C8FA0F4F023}">
   <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>